<commit_message>
test: repair supplier XLSX quote fixture
</commit_message>
<xml_diff>
--- a/tests/fixtures/rfq_quote_supplier_d.xlsx
+++ b/tests/fixtures/rfq_quote_supplier_d.xlsx
@@ -11,14 +11,14 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
     <row r="1">
-      <c r="A4" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Northstar Components Quote</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="2">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Quote Number: NS-4482</t>
         </is>

</xml_diff>